<commit_message>
feat: adiciona maturidade operacional e analytics financeiro
</commit_message>
<xml_diff>
--- a/reports/financial_report.xlsx
+++ b/reports/financial_report.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPCA Mensal" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotacoes B3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,6 +555,170 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Retorno nominal por ativo</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Performance'!F3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Performance'!$A$4:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Performance'!$F$4:$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Drawdown maximo por ativo</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Performance'!I3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Performance'!$A$4:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Performance'!$I$4:$I$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -627,6 +792,55 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -729,6 +943,26 @@
     <tableColumn id="12" name="first_adjusted_close"/>
     <tableColumn id="13" name="last_adjusted_close"/>
     <tableColumn id="14" name="return_pct"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_asset_performance" displayName="tbl_asset_performance" ref="A3:K6" headerRowCount="1">
+  <autoFilter ref="A3:K6"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="ticker"/>
+    <tableColumn id="2" name="start_date"/>
+    <tableColumn id="3" name="end_date"/>
+    <tableColumn id="4" name="initial_price"/>
+    <tableColumn id="5" name="final_price"/>
+    <tableColumn id="6" name="nominal_return_pct"/>
+    <tableColumn id="7" name="real_return_pct"/>
+    <tableColumn id="8" name="annualized_volatility_pct"/>
+    <tableColumn id="9" name="max_drawdown_pct"/>
+    <tableColumn id="10" name="benchmark_return_pct"/>
+    <tableColumn id="11" name="excess_return_pct"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1060,7 +1294,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28/06/2026 12:27:23</t>
+          <t>28/06/2026 13:02:36</t>
         </is>
       </c>
     </row>
@@ -40830,4 +41064,211 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Performance e Risco</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>initial_price</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>final_price</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>nominal_return_pct</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>real_return_pct</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>annualized_volatility_pct</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>max_drawdown_pct</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>benchmark_return_pct</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>excess_return_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>ITUB4.SA</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>45293</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>45656</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>23.82173919677734</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>23.42087173461914</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>-0.01682779997072725</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>-0.0621386556345338</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>0.1838066486798158</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>-0.1647727052437724</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>-0.09355147441162949</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>0.07672367444090224</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>PETR4.SA</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>45293</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>45656</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>26.84741592407227</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>31.51451110839844</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>0.1738377800502395</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>0.1197398364519604</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>0.2501656479142811</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>-0.1689977488447508</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-0.09355147441162949</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>0.267389254461869</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>VALE3.SA</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>45293</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>45656</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>62.31031799316406</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>48.19790267944336</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>-0.2264860101543528</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>-0.2621344761573456</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>0.2308839965329491</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>-0.2375463105925234</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-0.09355147441162949</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-0.1329345357427233</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona backfill historico e cobertura de dados
</commit_message>
<xml_diff>
--- a/reports/financial_report.xlsx
+++ b/reports/financial_report.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPCA Mensal" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotacoes B3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -567,6 +568,88 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Cobertura historica por dataset</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cobertura'!M3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cobertura'!$B$4:$B$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cobertura'!$M$4:$M$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Retorno nominal por ativo</a:t>
             </a:r>
           </a:p>
@@ -637,7 +720,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -804,6 +887,33 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>17</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>12</col>
       <colOff>0</colOff>
       <row>2</row>
@@ -949,7 +1059,32 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_asset_performance" displayName="tbl_asset_performance" ref="A3:K6" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_data_coverage" displayName="tbl_data_coverage" ref="A3:P11" headerRowCount="1">
+  <autoFilter ref="A3:P11"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="source_name"/>
+    <tableColumn id="2" name="dataset_name"/>
+    <tableColumn id="3" name="expected_frequency"/>
+    <tableColumn id="4" name="start_date"/>
+    <tableColumn id="5" name="end_date"/>
+    <tableColumn id="6" name="first_expected_date"/>
+    <tableColumn id="7" name="last_expected_date"/>
+    <tableColumn id="8" name="first_available_date"/>
+    <tableColumn id="9" name="last_available_date"/>
+    <tableColumn id="10" name="expected_observations"/>
+    <tableColumn id="11" name="actual_observations"/>
+    <tableColumn id="12" name="missing_observations"/>
+    <tableColumn id="13" name="coverage_pct"/>
+    <tableColumn id="14" name="status"/>
+    <tableColumn id="15" name="missing_sample"/>
+    <tableColumn id="16" name="generated_at"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_asset_performance" displayName="tbl_asset_performance" ref="A3:K6" headerRowCount="1">
   <autoFilter ref="A3:K6"/>
   <tableColumns count="11">
     <tableColumn id="1" name="ticker"/>
@@ -1294,7 +1429,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28/06/2026 13:02:36</t>
+          <t>28/06/2026 13:38:18</t>
         </is>
       </c>
     </row>
@@ -41072,6 +41207,716 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Cobertura Historica</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>dataset_name</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>expected_frequency</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>first_expected_date</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>last_expected_date</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>first_available_date</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>last_available_date</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>expected_observations</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>actual_observations</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>missing_observations</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>coverage_pct</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>missing_sample</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>generated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>BCB_SGS</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>cdi_daily</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>daily_business</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v/>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>BCB_SGS</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>ipca_monthly</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v/>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>BCB_SGS</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>selic_daily</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>daily_business</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v/>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>BCB_SGS</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>usd_brl_ptax_sell_daily</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>daily_business</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v/>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>ITUB4.SA</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>trading_day</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>251</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>0.9921</v>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-24, 2024-12-31</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>PETR4.SA</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>trading_day</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>251</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>0.9921</v>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-24, 2024-12-31</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>VALE3.SA</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>trading_day</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>251</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>0.9921</v>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-24, 2024-12-31</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>^BVSP</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>trading_day</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>251</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>0.9921</v>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-24, 2024-12-31</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 13:38:13</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
feat: adiciona fontes institucionais financeiras
</commit_message>
<xml_diff>
--- a/reports/financial_report.xlsx
+++ b/reports/financial_report.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundos CVM" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1059,9 +1060,9 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_data_coverage" displayName="tbl_data_coverage" ref="A3:P11" headerRowCount="1">
-  <autoFilter ref="A3:P11"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_data_coverage" displayName="tbl_data_coverage" ref="A3:R11" headerRowCount="1">
+  <autoFilter ref="A3:R11"/>
+  <tableColumns count="18">
     <tableColumn id="1" name="source_name"/>
     <tableColumn id="2" name="dataset_name"/>
     <tableColumn id="3" name="expected_frequency"/>
@@ -1076,8 +1077,10 @@
     <tableColumn id="12" name="missing_observations"/>
     <tableColumn id="13" name="coverage_pct"/>
     <tableColumn id="14" name="status"/>
-    <tableColumn id="15" name="missing_sample"/>
-    <tableColumn id="16" name="generated_at"/>
+    <tableColumn id="15" name="calendar_source"/>
+    <tableColumn id="16" name="last_expected_trading_date"/>
+    <tableColumn id="17" name="missing_sample"/>
+    <tableColumn id="18" name="generated_at"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1429,7 +1432,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28/06/2026 13:38:18</t>
+          <t>28/06/2026 14:13:54</t>
         </is>
       </c>
     </row>
@@ -41207,7 +41210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -41224,8 +41227,10 @@
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -41309,10 +41314,20 @@
       </c>
       <c r="O3" s="8" t="inlineStr">
         <is>
+          <t>calendar_source</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>last_expected_trading_date</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
           <t>missing_sample</t>
         </is>
       </c>
-      <c r="P3" s="8" t="inlineStr">
+      <c r="R3" s="8" t="inlineStr">
         <is>
           <t>generated_at</t>
         </is>
@@ -41381,12 +41396,22 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="O4" s="9" t="n">
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>brazil_business_day</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="n">
         <v/>
       </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-28 13:38:13</t>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41453,12 +41478,22 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="O5" s="9" t="n">
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>monthly_calendar</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="n">
         <v/>
       </c>
-      <c r="P5" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-28 13:38:13</t>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41525,12 +41560,22 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="O6" s="9" t="n">
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>brazil_business_day</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="n">
         <v/>
       </c>
-      <c r="P6" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-28 13:38:13</t>
+      <c r="R6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41597,12 +41642,22 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="O7" s="9" t="n">
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>brazil_business_day</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="n">
         <v/>
       </c>
-      <c r="P7" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-28 13:38:13</t>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41639,7 +41694,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2024-12-30</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
@@ -41653,16 +41708,16 @@
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>251</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>0.9921</v>
+        <v>1</v>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
@@ -41671,12 +41726,20 @@
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>2024-12-24, 2024-12-31</t>
+          <t>manual_reference</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-28 13:38:13</t>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="n">
+        <v/>
+      </c>
+      <c r="R8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41713,7 +41776,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2024-12-30</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -41727,16 +41790,16 @@
         </is>
       </c>
       <c r="J9" s="9" t="n">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>251</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>0.9921</v>
+        <v>1</v>
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
@@ -41745,12 +41808,20 @@
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>2024-12-24, 2024-12-31</t>
+          <t>manual_reference</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-28 13:38:13</t>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="n">
+        <v/>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41787,7 +41858,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2024-12-30</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -41801,16 +41872,16 @@
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>251</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>0.9921</v>
+        <v>1</v>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
@@ -41819,12 +41890,20 @@
       </c>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>2024-12-24, 2024-12-31</t>
+          <t>manual_reference</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-28 13:38:13</t>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v/>
+      </c>
+      <c r="R10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -41861,7 +41940,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2024-12-30</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
@@ -41875,16 +41954,16 @@
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>251</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>0.9921</v>
+        <v>1</v>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
@@ -41893,12 +41972,20 @@
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>2024-12-24, 2024-12-31</t>
+          <t>manual_reference</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-28 13:38:13</t>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v/>
+      </c>
+      <c r="R11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28 14:13:45</t>
         </is>
       </c>
     </row>
@@ -42116,4 +42203,43 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Fundos CVM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dados CVM nao carregados</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Execute python src\collect_data.py --include-cvm --cvm-year-month 202401 e depois a carga final.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>